<commit_message>
Atualização da página de papers e partners
</commit_message>
<xml_diff>
--- a/dados_site/colaboradores.xlsx
+++ b/dados_site/colaboradores.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -493,7 +493,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="n"/>
       <c r="B4" s="3" t="n"/>
@@ -569,6 +568,21 @@
           <t>ResearchGate</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Scholar</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Areas_Atuacao</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Universidade_Key</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -599,16 +613,26 @@
           <t>./assets/team/eugeniorodrigues.png</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="inlineStr">
         <is>
           <t>https://orcid.org/0000-0001-7023-4484</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="n"/>
       <c r="J7" s="4" t="inlineStr">
         <is>
           <t>https://www.researchgate.net/profile/Eugenio_Rodrigues</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Simulacao-Computacional, Mudancas-Climaticas</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>uc, cura-lab</t>
         </is>
       </c>
     </row>
@@ -641,16 +665,26 @@
           <t>./assets/team/andreateston.png</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="inlineStr">
         <is>
           <t>https://orcid.org/0000-0001-7529-382X</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="n"/>
       <c r="J8" s="4" t="inlineStr">
         <is>
           <t>https://www.researchgate.net/profile/Andrea-Teston</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Agua-Pluvial</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>udesc</t>
         </is>
       </c>
     </row>
@@ -683,14 +717,24 @@
           <t>./assets/team/matheusbbastos.png</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="inlineStr">
         <is>
           <t>https://orcid.org/0009-0006-7673-1338</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr"/>
-      <c r="J9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="n"/>
+      <c r="J9" s="4" t="n"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Simulacao-Computacional</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>ufsc-automacao</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -721,7 +765,7 @@
           <t>./assets/team/andresballarin.png</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="n"/>
       <c r="H10" s="4" t="inlineStr">
         <is>
           <t>https://orcid.org/0000-0001-6997-8662</t>
@@ -735,6 +779,16 @@
       <c r="J10" s="4" t="inlineStr">
         <is>
           <t>https://www.researchgate.net/profile/Andre-Ballarin</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Precipitacao</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>usp</t>
         </is>
       </c>
     </row>
@@ -744,37 +798,56 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Instituição Parceira</t>
+          <t>Colaborador</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Universidade Federal de Santa Catarina (UFSC)</t>
+          <t>Diego Custódio</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Programa de Pós-Graduação em Engenharia Civil</t>
+          <t>Pesquisador Colaborador</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>ufsc.png / ufsc_escuro.png</t>
+          <t>diegocustodio.jpg</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>./assets/logos/ufsc.png</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>https://ppgec.posgrad.ufsc.br/</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" s="4" t="inlineStr"/>
-      <c r="J11" s="4" t="inlineStr"/>
+          <t>./assets/team/diegocustodio.jpg</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-9777-7128</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>http://lattes.cnpq.br/4330940702408383</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="n"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?user=NtQbMaAAAAAJ&amp;hl=pt-BR</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Comportamento-Usuario, Conforto-Termico, Agua-Pluvial</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>utfpr</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -782,37 +855,55 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Instituição Parceira</t>
+          <t>Colaborador</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Universidade de Coimbra (UC)</t>
+          <t>Taylana Piccinini Scolaro</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Faculdade de Ciências e Tecnologia (FCTUC)</t>
+          <t>Pesquisadora Colaboradora</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>ftuc.png / ftuc_escuro.png</t>
+          <t>taylanapscolaro.png</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>./assets/logos/ftuc.png</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>https://www.uc.pt/fctuc</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr"/>
+          <t>./assets/team/taylanapscolaro.png</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0003-4296-0686</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>http://lattes.cnpq.br/7183244717269690</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.researchgate.net/profile/Taylana-Scolaro</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Mudancas-Climaticas, Simulacao-Computacional, Telhado-Verde</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>utfpr</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -825,32 +916,37 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Universidade de São Paulo (USP)</t>
+          <t>Universidade Federal de Santa Catarina (UFSC)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Escola de Engenharia de São Carlos (EESC)</t>
+          <t>Programa de Pós-Graduação em Engenharia Civil</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>uspsc.png / uspsc_escuro.png</t>
+          <t>ufsc.png / ufsc_escuro.png</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>./assets/logos/uspsc.png</t>
+          <t>./assets/logos/ufsc.png</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>https://eesc.usp.br/</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="4" t="inlineStr"/>
-      <c r="J13" s="4" t="inlineStr"/>
+          <t>https://ppgec.posgrad.ufsc.br/</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
+      <c r="J13" s="4" t="n"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>ufsc</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -863,32 +959,37 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Universidade do Estado de Santa Catarina (UDESC)</t>
+          <t>Universidade de Coimbra (UC)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Departamento de Arquitetura e Urbanismo</t>
+          <t>Faculdade de Ciências e Tecnologia (FCTUC)</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>udesc.png / udesc_escuro.png</t>
+          <t>ftuc.png / ftuc_escuro.png</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>./assets/logos/udesc.png</t>
+          <t>./assets/logos/ftuc.png</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>https://www.udesc.br/cct/dau</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr"/>
-      <c r="I14" s="4" t="inlineStr"/>
-      <c r="J14" s="4" t="inlineStr"/>
+          <t>https://www.uc.pt/fctuc</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>uc</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -901,32 +1002,37 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Universidade Federal de Mato Grosso do Sul (UFMS)</t>
+          <t>Universidade de São Paulo (USP)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Faculdade de Engenharia, Arquitetura e Urbanismo e Geografia</t>
+          <t>Escola de Engenharia de São Carlos (EESC)</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>UFMS.png / ufms_escuro.png</t>
+          <t>uspsc.png / uspsc_escuro.png</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>./assets/logos/UFMS.png</t>
+          <t>./assets/logos/uspsc.png</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>https://faeng.ufms.br/</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr"/>
-      <c r="I15" s="4" t="inlineStr"/>
-      <c r="J15" s="4" t="inlineStr"/>
+          <t>https://eesc.usp.br/</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="4" t="n"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>usp</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -939,32 +1045,157 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
+          <t>Universidade do Estado de Santa Catarina (UDESC)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Departamento de Arquitetura e Urbanismo</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>udesc.png / udesc_escuro.png</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>./assets/logos/udesc.png</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.udesc.br/cct/dau</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>udesc</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Instituição Parceira</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Universidade Federal de Mato Grosso do Sul (UFMS)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Faculdade de Engenharia, Arquitetura e Urbanismo e Geografia</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>UFMS.png / ufms_escuro.png</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>./assets/logos/UFMS.png</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://faeng.ufms.br/</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>ufms</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Instituição Parceira</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>Universidade Tecnológica Federal do Paraná (UTFPR)</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Universidade Parceira de Pesquisa</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Departamento de Engenharia Civil</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>UTFPR.png / UTFPR_escuro.png</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>./assets/logos/UTFPR.png</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>https://www.utfpr.edu.br/</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>utfpr</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Instituição Parceira</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CURA Lab (ADAI)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Laboratório de Pesquisa em Clima e Urbanismo</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>curalab.png</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>./assets/logos/curalab.png</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://cura-lab.adai.pt/</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>cura-lab</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Correção em problema em projetos e parceiros
</commit_message>
<xml_diff>
--- a/dados_site/colaboradores.xlsx
+++ b/dados_site/colaboradores.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -493,6 +493,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="n"/>
       <c r="B4" s="3" t="n"/>
@@ -1197,6 +1198,156 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Colaborador</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ricardo Forgiarini Rupp</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Pesquisador Colaborador</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ricardorupp.jpeg</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>./assets/team/ricardorupp.jpeg</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-8205-7259</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>http://lattes.cnpq.br/0355666000210770</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://www.researchgate.net/profile/Ricardo-Rupp</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Conforto-Termico, Comportamento-Usuario</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>denmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Colaborador</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Aldomar Pedrini</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Pesquisador Colaborador</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>aldomarpedrini.jpg</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>./assets/team/aldomarpedrini.jpg</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://orcid.org/0000-0002-6607-2176</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>http://lattes.cnpq.br/9012296636400514</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://www.researchgate.net/profile/Aldomar-Pedrini-2</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Conforto-Termico, Simulacao-Computacional</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>ufrn</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Instituição Parceira</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Universidade Federal do Rio Grande do Norte (UFRN)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Departamento de Arquitetura</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ufrn.png</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>./assets/logos/ufrn.png</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://ufrn.br/</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>ufrn</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>